<commit_message>
Revise ten-year Nifty takeaways and chart after fact and style review
Explain NSE's 2021 switch to consolidated earnings before relying on it,
use plain wording in the chart title, subtitle and legends, mark old-basis
values in the key strip, add PrimeInvestor's lower 1.05 ratio as a third
like-for-like case, correct verification counts and source dates, and widen
and space the three chart panels.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N5HxAwkVaTsKQoA79fMcaE
</commit_message>
<xml_diff>
--- a/analysis/nifty-decade/nifty_decade_price_pe_earnings.xlsx
+++ b/analysis/nifty-decade/nifty_decade_price_pe_earnings.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Method &amp; Sources" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Chart!$A$1:$V$52</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Chart!$A$1:$V$57</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -28,21 +28,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="204">
   <si>
-    <t xml:space="preserve">Until 2019 the Nifty rose on a rising P/E. Since then, earnings have done the lifting.</t>
+    <t xml:space="preserve">Until 2019, the Nifty rose because investors paid more for each rupee of profit. Since then, profits have done the lifting.</t>
   </si>
   <si>
-    <t xml:space="preserve">Over ten years the Nifty rose 2.6 times and its earnings 2.7 to 2.8 times (like-for-like), so its P/E ends a little below where it started.</t>
+    <t xml:space="preserve">Over ten years the Nifty grew 2.6 times and the profit behind it about 2.7 to 2.8 times, after adjusting for NSE's 2021 change in how profit is counted. So investors now pay the same or a little less for each rupee of profit as they did in 2016.</t>
   </si>
   <si>
-    <t xml:space="preserve">NSE switched from standalone to consolidated earnings on 31 Mar 2021, which cut its P/E from 40.4x to 33.2x overnight. Lighter lines show the old basis.</t>
+    <t xml:space="preserve">On 31 Mar 2021 NSE began counting subsidiaries' profits as well as the parent company's (consolidated instead of standalone earnings), which cut its P/E from 40.4x to 33.2x overnight. Lighter lines show the old method.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: NSE Indices (Nifty 50 P/E, trailing four quarters, month-end; via Downstox, checked against NSE Index Dashboards), Yahoo Finance (Nifty 50 daily closes). Earnings per unit = Nifty close ÷ NSE P/E. Data to 28 Sep 2026.</t>
+    <t xml:space="preserve">Source: NSE Indices (Nifty 50 P/E, trailing four quarters, month-end; via Downstox, checked against NSE Index Dashboards), Yahoo Finance (Nifty 50 daily closes). Profit per unit = Nifty close ÷ NSE P/E. Latest reading 28 Sep 2026.</t>
   </si>
   <si>
-    <t xml:space="preserve">Like-for-like: pre-2021 standalone earnings restated to a consolidated basis with a ratio of 1.14 (Bloomberg 10-year average) to 1.205 (NSE's switch day). Motilal Oswal's tally of actual Nifty EPS rose from ₹393 (FY16) to ₹1,065 (FY26), 2.7x.</t>
+    <t xml:space="preserve">* Old method (parent-company profit only). Changes in brackets are like-for-like: pre-2021 profit multiplied by 1.14 (Bloomberg's 10-year average gap) to 1.205 (the gap on NSE's switch day). A lower 2019 estimate of 1.05 (PrimeInvestor) would put the profit multiple at 3.1x. Motilal Oswal's separate count of Nifty EPS: ₹393 (FY16) to ₹1,065 (FY26), 2.7x.</t>
   </si>
   <si>
     <t xml:space="preserve">1 Finance | SEBI Registered Investment Advisor. This content is for information and educational purposes only. Please consult a Qualified Financial Advisor before making investment decisions.</t>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t xml:space="preserve">Default: the switch-day ratio. Type 1.14 (or anything else) to see how the like-for-like columns move.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low estimate, PrimeInvestor Dec 2019 (input)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PrimeInvestor: consolidated earnings "about 5 per cent higher than the standalone earnings"</t>
   </si>
   <si>
     <t xml:space="preserve">Point in time</t>
@@ -220,6 +226,9 @@
   </si>
   <si>
     <t xml:space="preserve">Measure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio 1.05 (PrimeInvestor, low)</t>
   </si>
   <si>
     <t xml:space="preserve">Ratio 1.14 (Bloomberg 10-yr average)</t>
@@ -459,16 +468,16 @@
     <t xml:space="preserve">31 Mar 2021, NSE switch day (this workbook, Summary!B9)</t>
   </si>
   <si>
-    <t xml:space="preserve">NSE P/E 40.43 (30 Mar, standalone) and 33.20 (31 Mar, consolidated)</t>
+    <t xml:space="preserve">NSE P/E 40.43 on 30 Mar (standalone) and 33.20 on 31 Mar (consolidated)</t>
   </si>
   <si>
     <t xml:space="preserve">https://downstox.com/nifty-pe/nifty-50</t>
   </si>
   <si>
-    <t xml:space="preserve">Dec 2020 (Bloomberg data)</t>
+    <t xml:space="preserve">Early 2021, earnings to Dec 2020 (Bloomberg data)</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hindu BusinessLine: "consolidated earnings of Nifty are about 16 per cent higher"</t>
+    <t xml:space="preserve">The Hindu BusinessLine (Mar 2021): "about 16 per cent higher"; the article's own figures (Rs 420 vs Rs 371) imply about 13%</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.thehindubusinessline.com/todays-paper/tp-investmentworld/article34010344.ece</t>
@@ -477,13 +486,22 @@
     <t xml:space="preserve">Average of the 10 years to 2020 (Bloomberg data)</t>
   </si>
   <si>
-    <t xml:space="preserve">The Hindu BusinessLine: "on the average ... 14 per cent higher"</t>
+    <t xml:space="preserve">The Hindu BusinessLine (Mar 2021): "on the average ... 14 per cent higher"</t>
   </si>
   <si>
     <t xml:space="preserve">Jan 2008 peak (P/E 26.5 standalone vs 23.3 consolidated)</t>
   </si>
   <si>
     <t xml:space="preserve">The Hindu BusinessLine (Bloomberg data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dec 2019 (low estimate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PrimeInvestor (Dec 2019): "consolidated earnings of the Nifty firms are about 5 per cent higher than the standalone earnings"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://primeinvestor.in/reports/what-they-dont-tell-you-about-the-nifty-pe/</t>
   </si>
   <si>
     <t xml:space="preserve">C. Actual Nifty EPS tallied by Motilal Oswal (fiscal years ending March) vs NSE-implied trailing EPS two months after year-end</t>
@@ -561,10 +579,10 @@
     <t xml:space="preserve">How this workbook was built</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Nifty 50 daily closes, 1 Sep 2016 to 28 Sep 2026, come from Yahoo Finance (^NSEI, NSE data). Every year was transcribed twice by independent agents and the two copies were diffed; all rows matched, and every month-end close matches Yahoo's monthly table. One missing day (29 Mar 2019) was filled from Yahoo's monthly table.</t>
+    <t xml:space="preserve">1. Nifty 50 daily closes, 1 Sep 2016 to 28 Sep 2026, come from Yahoo Finance (^NSEI, NSE data). Every year was transcribed twice by independent agents and the two copies were diffed: all 2,483 days in Yahoo's daily table matched, and every month-end close matches Yahoo's monthly table. The one missing day (29 Mar 2019) was filled from Yahoo's monthly table, making 2,484 days.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. NSE's Nifty 50 P/E (index market cap divided by trailing four-quarter earnings, as NSE Indices publishes it daily) is taken at each month-end from Downstox, which republishes NSE's series. 26 of these values were checked against NSE's own monthly Index Dashboards and Nippon India MF's daily notes; the largest gap was 0.08, which is Downstox's one-decimal rounding. September 2026 uses the 28 Sep 2026 reading (19.26).</t>
+    <t xml:space="preserve">2. NSE's Nifty 50 P/E (index market cap divided by trailing four-quarter earnings, as NSE Indices publishes it daily) is taken at each month-end from Downstox, which republishes NSE's series. 25 month-end values plus the 30 Mar 2021 daily reading were checked against NSE's own monthly Index Dashboards and Nippon India MF's notes; all but one agree within 0.05 (Downstox's one-decimal rounding) and the largest gap is 0.08 (Jul 2026, against a Nippon India product note). September 2026 uses the 28 Sep 2026 daily reading (19.26), not a month-end.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Earnings per unit = Nifty close / NSE P/E. This is NSE's trailing earnings for the index, as NSE counts them.</t>
@@ -573,7 +591,7 @@
     <t xml:space="preserve">4. On 31 Mar 2021 NSE switched from standalone to consolidated earnings. The P/E fell from 40.43 to 33.20 overnight while the index moved about 1%, so consolidated earnings were about 20.5% higher than standalone that day (Summary!B9).</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Like-for-like columns multiply pre-2021 earnings by a ratio (Summary!B11) to put them on a consolidated basis. The ratio was not constant: Bloomberg data put the 10-year average at 1.14 and Dec 2020 at 1.16, against 1.205 at NSE's switch. The Summary shows results at both ends of that range.</t>
+    <t xml:space="preserve">5. Like-for-like columns multiply pre-2021 earnings by a ratio (Summary!B11) to put them on a consolidated basis. The ratio changed over time: Bloomberg data put the 10-year average at 1.14 and early 2021 at about 1.13 to 1.16, NSE's switch day gave 1.205, and PrimeInvestor estimated only 1.05 in Dec 2019. The Summary shows results at 1.05, 1.14 and 1.205; the chart uses 1.14 to 1.205, the range best supported by NSE's own data and Bloomberg.</t>
   </si>
   <si>
     <t xml:space="preserve">6. Motilal Oswal's bottom-up tally of actual Nifty EPS (FY16 ₹393 to FY26 ₹1,065, 2.7x) is shown on the Validation sheet as an independent check.</t>
@@ -585,10 +603,10 @@
     <t xml:space="preserve">NSE's P/E is a trailing measure: it divides today's price by the last four quarters of reported profit. It is not the forward (expected-earnings) P/E that Bloomberg charts use, so its levels are higher; on 28 Sep 2026 NSE showed 19.3x while Bloomberg's forward P/E was about 17x.</t>
   </si>
   <si>
-    <t xml:space="preserve">Long-run "average Nifty P/E" figures quoted in the press (23x to 27x over 10 years) mostly mix the standalone and consolidated eras, so they overstate the average on today's basis. The consolidated-era median here is about 22x.</t>
+    <t xml:space="preserve">Some long-run "average Nifty P/E" figures (Business Standard 26.7x, Craytheon 23.28x over 10 years) include the higher standalone readings from before 2021, which makes today's P/E look further below normal than it is like-for-like. The consolidated-era median here is 22.0x.</t>
   </si>
   <si>
-    <t xml:space="preserve">The Nifty figures are the price index, without dividends. The total-return index grew about 1.3 percentage points a year faster over the ten years to July 2026 (NSE via Bajaj Finserv AMC).</t>
+    <t xml:space="preserve">The Nifty figures are the price index, without dividends. The total-return index grew about 1.35 percentage points a year faster over the ten years to 17 Jul 2026 (12.39% against 11.04% a year; NSE return profile via Bajaj Finserv AMC).</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -619,6 +637,9 @@
   </si>
   <si>
     <t xml:space="preserve">Nippon India MF (28 Sep 2026): Nifty 50 P/E 19.26.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PrimeInvestor (Dec 2019): consolidated Nifty earnings "about 5 per cent higher than the standalone earnings".</t>
   </si>
 </sst>
 </file>
@@ -670,7 +691,7 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="20"/>
+      <sz val="17"/>
       <color rgb="FF272623"/>
       <name val="Fira Sans"/>
       <family val="0"/>
@@ -903,8 +924,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -919,12 +940,12 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -16028,11 +16049,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="96687625"/>
-        <c:axId val="6840256"/>
+        <c:axId val="13914200"/>
+        <c:axId val="97023733"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="96687625"/>
+        <c:axId val="13914200"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="46296"/>
@@ -16066,13 +16087,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6840256"/>
+        <c:crossAx val="97023733"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="365.25"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="6840256"/>
+        <c:axId val="97023733"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="30000"/>
@@ -16147,7 +16168,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96687625"/>
+        <c:crossAx val="13914200"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="5000"/>
@@ -16212,11 +16233,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"Earnings per unit, standalone basis (to Feb 2021)"</c:f>
+              <c:f>"Profit per unit, old method: parent company only (to Feb 2021)"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Earnings per unit, standalone basis (to Feb 2021)</c:v>
+                  <c:v>Profit per unit, old method: parent company only (to Feb 2021)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -16609,11 +16630,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"Consolidated basis (from Mar 2021)"</c:f>
+              <c:f>"New method, with subsidiaries (from Mar 2021)"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Consolidated basis (from Mar 2021)</c:v>
+                  <c:v>New method, with subsidiaries (from Mar 2021)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -17113,11 +17134,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="13344925"/>
-        <c:axId val="58540505"/>
+        <c:axId val="19770977"/>
+        <c:axId val="24710225"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="13344925"/>
+        <c:axId val="19770977"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="46296"/>
@@ -17151,13 +17172,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58540505"/>
+        <c:crossAx val="24710225"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="365.25"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="58540505"/>
+        <c:axId val="24710225"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1400"/>
@@ -17196,7 +17217,7 @@
                     </a:solidFill>
                     <a:latin typeface="Fira Sans"/>
                   </a:rPr>
-                  <a:t>Trailing earnings (₹)</a:t>
+                  <a:t>Profit per unit, last 4 quarters (₹)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -17232,7 +17253,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13344925"/>
+        <c:crossAx val="19770977"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="200"/>
@@ -17297,11 +17318,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>"NSE P/E, standalone earnings (to Feb 2021)"</c:f>
+              <c:f>"NSE P/E, old method (to Feb 2021)"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>NSE P/E, standalone earnings (to Feb 2021)</c:v>
+                  <c:v>NSE P/E, old method (to Feb 2021)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -17694,11 +17715,11 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>"Consolidated earnings (from Mar 2021)"</c:f>
+              <c:f>"New method (from Mar 2021)"</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Consolidated earnings (from Mar 2021)</c:v>
+                  <c:v>New method (from Mar 2021)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -18254,7 +18275,7 @@
           </c:dLbls>
           <c:xVal>
             <c:numRef>
-              <c:f>Summary!$A$49:$A$50</c:f>
+              <c:f>Summary!$A$50:$A$51</c:f>
               <c:numCache>
                 <c:formatCode>dd\-mmm\-yyyy</c:formatCode>
                 <c:ptCount val="2"/>
@@ -18269,7 +18290,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Summary!$B$49:$B$50</c:f>
+              <c:f>Summary!$B$50:$B$51</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
@@ -18284,11 +18305,11 @@
           </c:yVal>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="26048834"/>
-        <c:axId val="93252343"/>
+        <c:axId val="90845500"/>
+        <c:axId val="6137255"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="26048834"/>
+        <c:axId val="90845500"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="46296"/>
@@ -18322,13 +18343,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="93252343"/>
+        <c:crossAx val="6137255"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="365.25"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="93252343"/>
+        <c:axId val="6137255"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="45"/>
@@ -18367,7 +18388,7 @@
                     </a:solidFill>
                     <a:latin typeface="Fira Sans"/>
                   </a:rPr>
-                  <a:t>NSE trailing P/E</a:t>
+                  <a:t>NSE P/E (trailing)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -18403,7 +18424,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26048834"/>
+        <c:crossAx val="90845500"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="5"/>
@@ -18463,10 +18484,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>378360</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>172080</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>57960</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -18474,8 +18495,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="222120" y="1562040"/>
-        <a:ext cx="10619640" cy="2267640"/>
+        <a:off x="222120" y="1866960"/>
+        <a:ext cx="13499640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -18489,14 +18510,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>378360</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>172080</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>57960</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>42840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -18504,8 +18525,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="222120" y="4038480"/>
-        <a:ext cx="10619640" cy="2267640"/>
+        <a:off x="222120" y="4724280"/>
+        <a:ext cx="13499640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -18519,14 +18540,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>378360</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>172440</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>57960</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>43200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -18534,8 +18555,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="222120" y="6515280"/>
-        <a:ext cx="10619640" cy="2267640"/>
+        <a:off x="222120" y="7581960"/>
+        <a:ext cx="13499640" cy="2519640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -18765,7 +18786,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:Q51"/>
+  <dimension ref="B1:V56"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2.5"/>
@@ -18778,51 +18799,173 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="str">
-        <f aca="false">"Nifty 50   "&amp;TEXT(Summary!C14,"#,##0")&amp;"  →  "&amp;TEXT(Summary!C21,"#,##0")&amp;"   ("&amp;TEXT(Summary!I14,"0.0")&amp;"x)"</f>
+        <f aca="false">"Nifty 50   "&amp;TEXT(Summary!C15,"#,##0")&amp;"  →  "&amp;TEXT(Summary!C22,"#,##0")&amp;"   ("&amp;TEXT(Summary!I15,"0.0")&amp;"x)"</f>
         <v>Nifty 50   8,611  →  22,780   (2.6x)</v>
       </c>
       <c r="I6" s="4" t="str">
-        <f aca="false">"Earnings per unit   ₹"&amp;TEXT(Summary!F14,"#,##0")&amp;"  →  ₹"&amp;TEXT(Summary!F21,"#,##0")&amp;"   ("&amp;TEXT(Summary!C33,"0.0")&amp;"x to "&amp;TEXT(Summary!B33,"0.0")&amp;"x like-for-like)"</f>
-        <v>Earnings per unit   ₹368  →  ₹1,183   (2.7x to 2.8x like-for-like)</v>
+        <f aca="false">"Profit per unit   ₹"&amp;TEXT(Summary!F15,"#,##0")&amp;"*  →  ₹"&amp;TEXT(Summary!F22,"#,##0")&amp;"   ("&amp;TEXT(Summary!D34,"0.0")&amp;"x to "&amp;TEXT(Summary!C34,"0.0")&amp;"x)"</f>
+        <v>Profit per unit   ₹368*  →  ₹1,183   (2.7x to 2.8x)</v>
       </c>
       <c r="Q6" s="5" t="str">
-        <f aca="false">"NSE P/E   "&amp;TEXT(Summary!D14,"0.0")&amp;"x  →  "&amp;TEXT(Summary!D21,"0.0")&amp;"x"</f>
-        <v>NSE P/E   23.4x  →  19.3x</v>
+        <f aca="false">"P/E   "&amp;TEXT(Summary!D15,"0.0")&amp;"x*  →  "&amp;TEXT(Summary!D22,"0.0")&amp;"x   ("&amp;TEXT(Summary!D36,"+0%;-0%")&amp;" to "&amp;TEXT(Summary!C36,"+0%;-0%")&amp;")"</f>
+        <v>P/E   23.4x*  →  19.3x   (-1% to -6%)</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="6" t="s">
+    <row r="53" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="6" t="s">
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+      <c r="H53" s="6"/>
+      <c r="I53" s="6"/>
+      <c r="J53" s="6"/>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" s="6"/>
+      <c r="N53" s="6"/>
+      <c r="O53" s="6"/>
+      <c r="P53" s="6"/>
+      <c r="Q53" s="6"/>
+      <c r="R53" s="6"/>
+      <c r="S53" s="6"/>
+      <c r="T53" s="6"/>
+      <c r="U53" s="6"/>
+      <c r="V53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="6" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="6"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="7" t="s">
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="6"/>
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="6"/>
+      <c r="N54" s="6"/>
+      <c r="O54" s="6"/>
+      <c r="P54" s="6"/>
+      <c r="Q54" s="6"/>
+      <c r="R54" s="6"/>
+      <c r="S54" s="6"/>
+      <c r="T54" s="6"/>
+      <c r="U54" s="6"/>
+      <c r="V54" s="6"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="6"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+      <c r="J55" s="6"/>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+      <c r="M55" s="6"/>
+      <c r="N55" s="6"/>
+      <c r="O55" s="6"/>
+      <c r="P55" s="6"/>
+      <c r="Q55" s="6"/>
+      <c r="R55" s="6"/>
+      <c r="S55" s="6"/>
+      <c r="T55" s="6"/>
+      <c r="U55" s="6"/>
+      <c r="V55" s="6"/>
+    </row>
+    <row r="56" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="7" t="s">
         <v>5</v>
       </c>
+      <c r="C56" s="7"/>
+      <c r="D56" s="7"/>
+      <c r="E56" s="7"/>
+      <c r="F56" s="7"/>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+      <c r="J56" s="7"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="7"/>
+      <c r="M56" s="7"/>
+      <c r="N56" s="7"/>
+      <c r="O56" s="7"/>
+      <c r="P56" s="7"/>
+      <c r="Q56" s="7"/>
+      <c r="R56" s="7"/>
+      <c r="S56" s="7"/>
+      <c r="T56" s="7"/>
+      <c r="U56" s="7"/>
+      <c r="V56" s="7"/>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B3:S3"/>
+    <mergeCell ref="B4:S4"/>
+    <mergeCell ref="B53:V53"/>
+    <mergeCell ref="B54:V54"/>
+    <mergeCell ref="B55:V55"/>
+    <mergeCell ref="B56:V56"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -42515,7 +42658,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
@@ -42603,101 +42746,67 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="30" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B12" s="28" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="30" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="B14" s="30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="E13" s="30" t="s">
-        <v>36</v>
-      </c>
-      <c r="F13" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="G13" s="30" t="s">
+      <c r="E14" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="F14" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="I13" s="30" t="s">
+      <c r="G14" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="J13" s="30" t="s">
+      <c r="H14" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="K13" s="30" t="s">
+      <c r="I14" s="30" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="s">
+      <c r="J14" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="32" t="n">
+      <c r="K14" s="30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="31" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="32" t="n">
         <f aca="false">INDEX(Monthly!$A:$A,2)</f>
         <v>42643</v>
       </c>
-      <c r="C14" s="10" t="n">
-        <f aca="false">INDEX(Monthly!$B:$B,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>8611.15</v>
-      </c>
-      <c r="D14" s="33" t="n">
-        <f aca="false">INDEX(Monthly!$C:$C,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>23.4</v>
-      </c>
-      <c r="E14" s="24" t="str">
-        <f aca="false">INDEX(Monthly!$D:$D,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>standalone</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <f aca="false">INDEX(Monthly!$E:$E,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>367.997863247863</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <f aca="false">INDEX(Monthly!$F:$F,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>443.476199673265</v>
-      </c>
-      <c r="H14" s="33" t="n">
-        <f aca="false">INDEX(Monthly!$G:$G,MATCH($B14,Monthly!$A:$A,0))</f>
-        <v>19.4173892676639</v>
-      </c>
-      <c r="I14" s="34" t="n">
-        <f aca="false">$C$21/C14</f>
-        <v>2.64543643996447</v>
-      </c>
-      <c r="J14" s="34" t="n">
-        <f aca="false">$G$21/G14</f>
-        <v>2.66705447235996</v>
-      </c>
-      <c r="K14" s="34" t="n">
-        <f aca="false">$H$21/H14</f>
-        <v>0.991894416623456</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2019,12,31),Monthly!$A:$A,1))</f>
-        <v>43830</v>
-      </c>
       <c r="C15" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B15,Monthly!$A:$A,0))</f>
-        <v>12168.45</v>
+        <v>8611.15</v>
       </c>
       <c r="D15" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B15,Monthly!$A:$A,0))</f>
-        <v>28.3</v>
+        <v>23.4</v>
       </c>
       <c r="E15" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B15,Monthly!$A:$A,0))</f>
@@ -42705,44 +42814,44 @@
       </c>
       <c r="F15" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B15,Monthly!$A:$A,0))</f>
-        <v>429.980565371025</v>
+        <v>367.997863247863</v>
       </c>
       <c r="G15" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B15,Monthly!$A:$A,0))</f>
-        <v>518.171886600515</v>
+        <v>443.476199673265</v>
       </c>
       <c r="H15" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B15,Monthly!$A:$A,0))</f>
-        <v>23.4834237724311</v>
+        <v>19.4173892676639</v>
       </c>
       <c r="I15" s="34" t="n">
-        <f aca="false">$C$21/C15</f>
-        <v>1.8720749150467</v>
+        <f aca="false">$C$22/C15</f>
+        <v>2.64543643996447</v>
       </c>
       <c r="J15" s="34" t="n">
-        <f aca="false">$G$21/G15</f>
-        <v>2.28259234495221</v>
+        <f aca="false">$G$22/G15</f>
+        <v>2.66705447235996</v>
       </c>
       <c r="K15" s="34" t="n">
-        <f aca="false">$H$21/H15</f>
-        <v>0.820152980529642</v>
+        <f aca="false">$H$22/H15</f>
+        <v>0.991894416623456</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2020,3,31),Monthly!$A:$A,1))</f>
-        <v>43921</v>
+        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2019,12,31),Monthly!$A:$A,1))</f>
+        <v>43830</v>
       </c>
       <c r="C16" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B16,Monthly!$A:$A,0))</f>
-        <v>8597.75</v>
+        <v>12168.45</v>
       </c>
       <c r="D16" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B16,Monthly!$A:$A,0))</f>
-        <v>19.4</v>
+        <v>28.3</v>
       </c>
       <c r="E16" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B16,Monthly!$A:$A,0))</f>
@@ -42750,44 +42859,44 @@
       </c>
       <c r="F16" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B16,Monthly!$A:$A,0))</f>
-        <v>443.182989690722</v>
+        <v>429.980565371025</v>
       </c>
       <c r="G16" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B16,Monthly!$A:$A,0))</f>
-        <v>534.082198992274</v>
+        <v>518.171886600515</v>
       </c>
       <c r="H16" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B16,Monthly!$A:$A,0))</f>
-        <v>16.0981774270376</v>
+        <v>23.4834237724311</v>
       </c>
       <c r="I16" s="34" t="n">
-        <f aca="false">$C$21/C16</f>
-        <v>2.64955947777035</v>
+        <f aca="false">$C$22/C16</f>
+        <v>1.8720749150467</v>
       </c>
       <c r="J16" s="34" t="n">
-        <f aca="false">$G$21/G16</f>
-        <v>2.21459390325213</v>
+        <f aca="false">$G$22/G16</f>
+        <v>2.28259234495221</v>
       </c>
       <c r="K16" s="34" t="n">
-        <f aca="false">$H$21/H16</f>
-        <v>1.19640872932932</v>
+        <f aca="false">$H$22/H16</f>
+        <v>0.820152980529642</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B17" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2021,2,28),Monthly!$A:$A,1))</f>
-        <v>44253</v>
+        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2020,3,31),Monthly!$A:$A,1))</f>
+        <v>43921</v>
       </c>
       <c r="C17" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B17,Monthly!$A:$A,0))</f>
-        <v>14529.15</v>
+        <v>8597.75</v>
       </c>
       <c r="D17" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B17,Monthly!$A:$A,0))</f>
-        <v>39.6</v>
+        <v>19.4</v>
       </c>
       <c r="E17" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B17,Monthly!$A:$A,0))</f>
@@ -42795,89 +42904,89 @@
       </c>
       <c r="F17" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B17,Monthly!$A:$A,0))</f>
-        <v>366.897727272727</v>
+        <v>443.182989690722</v>
       </c>
       <c r="G17" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B17,Monthly!$A:$A,0))</f>
-        <v>442.150419906308</v>
+        <v>534.082198992274</v>
       </c>
       <c r="H17" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B17,Monthly!$A:$A,0))</f>
-        <v>32.8601972222004</v>
+        <v>16.0981774270376</v>
       </c>
       <c r="I17" s="34" t="n">
-        <f aca="false">$C$21/C17</f>
-        <v>1.56789970507566</v>
+        <f aca="false">$C$22/C17</f>
+        <v>2.64955947777035</v>
       </c>
       <c r="J17" s="34" t="n">
-        <f aca="false">$G$21/G17</f>
-        <v>2.67505158532793</v>
+        <f aca="false">$G$22/G17</f>
+        <v>2.21459390325213</v>
       </c>
       <c r="K17" s="34" t="n">
-        <f aca="false">$H$21/H17</f>
-        <v>0.58611942800477</v>
+        <f aca="false">$H$22/H17</f>
+        <v>1.19640872932932</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B18" s="32" t="n">
+        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2021,2,28),Monthly!$A:$A,1))</f>
+        <v>44253</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <f aca="false">INDEX(Monthly!$B:$B,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>14529.15</v>
+      </c>
+      <c r="D18" s="33" t="n">
+        <f aca="false">INDEX(Monthly!$C:$C,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>39.6</v>
+      </c>
+      <c r="E18" s="24" t="str">
+        <f aca="false">INDEX(Monthly!$D:$D,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>standalone</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <f aca="false">INDEX(Monthly!$E:$E,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>366.897727272727</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <f aca="false">INDEX(Monthly!$F:$F,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>442.150419906308</v>
+      </c>
+      <c r="H18" s="33" t="n">
+        <f aca="false">INDEX(Monthly!$G:$G,MATCH($B18,Monthly!$A:$A,0))</f>
+        <v>32.8601972222004</v>
+      </c>
+      <c r="I18" s="34" t="n">
+        <f aca="false">$C$22/C18</f>
+        <v>1.56789970507566</v>
+      </c>
+      <c r="J18" s="34" t="n">
+        <f aca="false">$G$22/G18</f>
+        <v>2.67505158532793</v>
+      </c>
+      <c r="K18" s="34" t="n">
+        <f aca="false">$H$22/H18</f>
+        <v>0.58611942800477</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="31" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="32" t="n">
         <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2021,3,31),Monthly!$A:$A,1))</f>
         <v>44286</v>
       </c>
-      <c r="C18" s="10" t="n">
-        <f aca="false">INDEX(Monthly!$B:$B,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>14690.7</v>
-      </c>
-      <c r="D18" s="33" t="n">
-        <f aca="false">INDEX(Monthly!$C:$C,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>33.2</v>
-      </c>
-      <c r="E18" s="24" t="str">
-        <f aca="false">INDEX(Monthly!$D:$D,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>consolidated</v>
-      </c>
-      <c r="F18" s="13" t="n">
-        <f aca="false">INDEX(Monthly!$E:$E,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>442.490963855422</v>
-      </c>
-      <c r="G18" s="13" t="n">
-        <f aca="false">INDEX(Monthly!$F:$F,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>442.490963855422</v>
-      </c>
-      <c r="H18" s="33" t="n">
-        <f aca="false">INDEX(Monthly!$G:$G,MATCH($B18,Monthly!$A:$A,0))</f>
-        <v>33.2</v>
-      </c>
-      <c r="I18" s="34" t="n">
-        <f aca="false">$C$21/C18</f>
-        <v>1.55065789921515</v>
-      </c>
-      <c r="J18" s="34" t="n">
-        <f aca="false">$G$21/G18</f>
-        <v>2.67299284807596</v>
-      </c>
-      <c r="K18" s="34" t="n">
-        <f aca="false">$H$21/H18</f>
-        <v>0.580120481927711</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="31" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2024,9,30),Monthly!$A:$A,1))</f>
-        <v>45565</v>
-      </c>
       <c r="C19" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B19,Monthly!$A:$A,0))</f>
-        <v>25810.85</v>
+        <v>14690.7</v>
       </c>
       <c r="D19" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B19,Monthly!$A:$A,0))</f>
-        <v>24.3</v>
+        <v>33.2</v>
       </c>
       <c r="E19" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B19,Monthly!$A:$A,0))</f>
@@ -42885,44 +42994,44 @@
       </c>
       <c r="F19" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B19,Monthly!$A:$A,0))</f>
-        <v>1062.17489711934</v>
+        <v>442.490963855422</v>
       </c>
       <c r="G19" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B19,Monthly!$A:$A,0))</f>
-        <v>1062.17489711934</v>
+        <v>442.490963855422</v>
       </c>
       <c r="H19" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B19,Monthly!$A:$A,0))</f>
-        <v>24.3</v>
+        <v>33.2</v>
       </c>
       <c r="I19" s="34" t="n">
-        <f aca="false">$C$21/C19</f>
-        <v>0.882584262044838</v>
+        <f aca="false">$C$22/C19</f>
+        <v>1.55065789921515</v>
       </c>
       <c r="J19" s="34" t="n">
-        <f aca="false">$G$21/G19</f>
-        <v>1.11354089136498</v>
+        <f aca="false">$G$22/G19</f>
+        <v>2.67299284807596</v>
       </c>
       <c r="K19" s="34" t="n">
-        <f aca="false">$H$21/H19</f>
-        <v>0.792592592592593</v>
+        <f aca="false">$H$22/H19</f>
+        <v>0.580120481927711</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2025,12,31),Monthly!$A:$A,1))</f>
-        <v>46022</v>
+        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2024,9,30),Monthly!$A:$A,1))</f>
+        <v>45565</v>
       </c>
       <c r="C20" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B20,Monthly!$A:$A,0))</f>
-        <v>26129.6</v>
+        <v>25810.85</v>
       </c>
       <c r="D20" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B20,Monthly!$A:$A,0))</f>
-        <v>22.75</v>
+        <v>24.3</v>
       </c>
       <c r="E20" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B20,Monthly!$A:$A,0))</f>
@@ -42930,44 +43039,44 @@
       </c>
       <c r="F20" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B20,Monthly!$A:$A,0))</f>
-        <v>1148.55384615385</v>
+        <v>1062.17489711934</v>
       </c>
       <c r="G20" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B20,Monthly!$A:$A,0))</f>
-        <v>1148.55384615385</v>
+        <v>1062.17489711934</v>
       </c>
       <c r="H20" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B20,Monthly!$A:$A,0))</f>
-        <v>22.75</v>
+        <v>24.3</v>
       </c>
       <c r="I20" s="34" t="n">
-        <f aca="false">$C$21/C20</f>
-        <v>0.871817785193803</v>
+        <f aca="false">$C$22/C20</f>
+        <v>0.882584262044838</v>
       </c>
       <c r="J20" s="34" t="n">
-        <f aca="false">$G$21/G20</f>
-        <v>1.02979515125436</v>
+        <f aca="false">$G$22/G20</f>
+        <v>1.11354089136498</v>
       </c>
       <c r="K20" s="34" t="n">
-        <f aca="false">$H$21/H20</f>
-        <v>0.846593406593407</v>
+        <f aca="false">$H$22/H20</f>
+        <v>0.792592592592593</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="35" t="s">
-        <v>50</v>
+      <c r="A21" s="31" t="s">
+        <v>51</v>
       </c>
       <c r="B21" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A:$A,122)</f>
-        <v>46293</v>
+        <f aca="false">INDEX(Monthly!$A:$A,MATCH(DATE(2025,12,31),Monthly!$A:$A,1))</f>
+        <v>46022</v>
       </c>
       <c r="C21" s="10" t="n">
         <f aca="false">INDEX(Monthly!$B:$B,MATCH($B21,Monthly!$A:$A,0))</f>
-        <v>22780.25</v>
+        <v>26129.6</v>
       </c>
       <c r="D21" s="33" t="n">
         <f aca="false">INDEX(Monthly!$C:$C,MATCH($B21,Monthly!$A:$A,0))</f>
-        <v>19.26</v>
+        <v>22.75</v>
       </c>
       <c r="E21" s="24" t="str">
         <f aca="false">INDEX(Monthly!$D:$D,MATCH($B21,Monthly!$A:$A,0))</f>
@@ -42975,343 +43084,423 @@
       </c>
       <c r="F21" s="13" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH($B21,Monthly!$A:$A,0))</f>
-        <v>1182.77518172378</v>
+        <v>1148.55384615385</v>
       </c>
       <c r="G21" s="13" t="n">
         <f aca="false">INDEX(Monthly!$F:$F,MATCH($B21,Monthly!$A:$A,0))</f>
-        <v>1182.77518172378</v>
+        <v>1148.55384615385</v>
       </c>
       <c r="H21" s="33" t="n">
         <f aca="false">INDEX(Monthly!$G:$G,MATCH($B21,Monthly!$A:$A,0))</f>
+        <v>22.75</v>
+      </c>
+      <c r="I21" s="34" t="n">
+        <f aca="false">$C$22/C21</f>
+        <v>0.871817785193803</v>
+      </c>
+      <c r="J21" s="34" t="n">
+        <f aca="false">$G$22/G21</f>
+        <v>1.02979515125436</v>
+      </c>
+      <c r="K21" s="34" t="n">
+        <f aca="false">$H$22/H21</f>
+        <v>0.846593406593407</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="32" t="n">
+        <f aca="false">INDEX(Monthly!$A:$A,122)</f>
+        <v>46293</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <f aca="false">INDEX(Monthly!$B:$B,MATCH($B22,Monthly!$A:$A,0))</f>
+        <v>22780.25</v>
+      </c>
+      <c r="D22" s="33" t="n">
+        <f aca="false">INDEX(Monthly!$C:$C,MATCH($B22,Monthly!$A:$A,0))</f>
         <v>19.26</v>
       </c>
-      <c r="I21" s="34" t="n">
-        <f aca="false">$C$21/C21</f>
+      <c r="E22" s="24" t="str">
+        <f aca="false">INDEX(Monthly!$D:$D,MATCH($B22,Monthly!$A:$A,0))</f>
+        <v>consolidated</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <f aca="false">INDEX(Monthly!$E:$E,MATCH($B22,Monthly!$A:$A,0))</f>
+        <v>1182.77518172378</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <f aca="false">INDEX(Monthly!$F:$F,MATCH($B22,Monthly!$A:$A,0))</f>
+        <v>1182.77518172378</v>
+      </c>
+      <c r="H22" s="33" t="n">
+        <f aca="false">INDEX(Monthly!$G:$G,MATCH($B22,Monthly!$A:$A,0))</f>
+        <v>19.26</v>
+      </c>
+      <c r="I22" s="34" t="n">
+        <f aca="false">$C$22/C22</f>
         <v>1</v>
       </c>
-      <c r="J21" s="34" t="n">
-        <f aca="false">$G$21/G21</f>
+      <c r="J22" s="34" t="n">
+        <f aca="false">$G$22/G22</f>
         <v>1</v>
       </c>
-      <c r="K21" s="34" t="n">
-        <f aca="false">$H$21/H21</f>
+      <c r="K22" s="34" t="n">
+        <f aca="false">$H$22/H22</f>
         <v>1</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" s="36" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="36" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="36" t="s">
+      <c r="B25" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="36" t="s">
+      <c r="C25" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="F24" s="36" t="s">
+      <c r="D25" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="36" t="s">
+      <c r="E25" s="36" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="31" t="s">
+      <c r="F25" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="32" t="n">
-        <f aca="false">B14</f>
-        <v>42643</v>
-      </c>
-      <c r="C25" s="32" t="n">
-        <f aca="false">B15</f>
-        <v>43830</v>
-      </c>
-      <c r="D25" s="37" t="n">
-        <f aca="false">C15/C14-1</f>
-        <v>0.413103940820913</v>
-      </c>
-      <c r="E25" s="37" t="n">
-        <f aca="false">F15/F14-1</f>
-        <v>0.16843223375298</v>
-      </c>
-      <c r="F25" s="37" t="n">
-        <f aca="false">D15/D14-1</f>
-        <v>0.20940170940171</v>
-      </c>
-      <c r="G25" s="38" t="n">
-        <f aca="false">(C15/C14)^(365.25/(B15-B14))-1</f>
-        <v>0.11226904484714</v>
+      <c r="G25" s="36" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B26" s="32" t="n">
         <f aca="false">B15</f>
+        <v>42643</v>
+      </c>
+      <c r="C26" s="32" t="n">
+        <f aca="false">B16</f>
         <v>43830</v>
       </c>
-      <c r="C26" s="32" t="n">
-        <f aca="false">B21</f>
-        <v>46293</v>
-      </c>
       <c r="D26" s="37" t="n">
-        <f aca="false">C21/C15-1</f>
-        <v>0.872074915046698</v>
+        <f aca="false">C16/C15-1</f>
+        <v>0.413103940820913</v>
       </c>
       <c r="E26" s="37" t="n">
-        <f aca="false">F21/F15-1</f>
-        <v>1.75076428327215</v>
+        <f aca="false">F16/F15-1</f>
+        <v>0.16843223375298</v>
       </c>
       <c r="F26" s="37" t="n">
-        <f aca="false">D21/D15-1</f>
-        <v>-0.319434628975265</v>
+        <f aca="false">D16/D15-1</f>
+        <v>0.20940170940171</v>
       </c>
       <c r="G26" s="38" t="n">
-        <f aca="false">(C21/C15)^(365.25/(B21-B15))-1</f>
-        <v>0.0974483953209322</v>
+        <f aca="false">(C16/C15)^(365.25/(B16-B15))-1</f>
+        <v>0.11226904484714</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="31" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B27" s="32" t="n">
-        <f aca="false">B14</f>
+        <f aca="false">B16</f>
+        <v>43830</v>
+      </c>
+      <c r="C27" s="32" t="n">
+        <f aca="false">B22</f>
+        <v>46293</v>
+      </c>
+      <c r="D27" s="37" t="n">
+        <f aca="false">C22/C16-1</f>
+        <v>0.872074915046698</v>
+      </c>
+      <c r="E27" s="37" t="n">
+        <f aca="false">F22/F16-1</f>
+        <v>1.75076428327215</v>
+      </c>
+      <c r="F27" s="37" t="n">
+        <f aca="false">D22/D16-1</f>
+        <v>-0.319434628975265</v>
+      </c>
+      <c r="G27" s="38" t="n">
+        <f aca="false">(C22/C16)^(365.25/(B22-B16))-1</f>
+        <v>0.0974483953209322</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="31" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="32" t="n">
+        <f aca="false">B15</f>
         <v>42643</v>
       </c>
-      <c r="C27" s="32" t="n">
-        <f aca="false">B21</f>
+      <c r="C28" s="32" t="n">
+        <f aca="false">B22</f>
         <v>46293</v>
       </c>
-      <c r="D27" s="37" t="n">
-        <f aca="false">C21/C14-1</f>
+      <c r="D28" s="37" t="n">
+        <f aca="false">C22/C15-1</f>
         <v>1.64543643996447</v>
       </c>
-      <c r="E27" s="37" t="n">
-        <f aca="false">F21/F14-1</f>
+      <c r="E28" s="37" t="n">
+        <f aca="false">F22/F15-1</f>
         <v>2.21408165603159</v>
       </c>
-      <c r="F27" s="37" t="n">
-        <f aca="false">D21/D14-1</f>
+      <c r="F28" s="37" t="n">
+        <f aca="false">D22/D15-1</f>
         <v>-0.176923076923077</v>
       </c>
-      <c r="G27" s="38" t="n">
-        <f aca="false">(C21/C14)^(365.25/(B21-B14))-1</f>
+      <c r="G28" s="38" t="n">
+        <f aca="false">(C22/C15)^(365.25/(B22-B15))-1</f>
         <v>0.102246354960462</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="B31" s="36" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="36" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="36" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="24" t="s">
+      <c r="B32" s="36" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="39" t="n">
+      <c r="C32" s="36" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="36" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" s="39" t="n">
+        <f aca="false">$B$12</f>
+        <v>1.05</v>
+      </c>
+      <c r="C33" s="39" t="n">
         <f aca="false">$B$10</f>
         <v>1.14</v>
       </c>
-      <c r="C32" s="39" t="n">
+      <c r="D33" s="39" t="n">
         <f aca="false">$B$9</f>
         <v>1.20510536599111</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="34" t="n">
-        <f aca="false">$F$21/($F$14*$B$32)</f>
-        <v>2.81936987371192</v>
-      </c>
-      <c r="C33" s="34" t="n">
-        <f aca="false">$F$21/($F$14*$C$32)</f>
-        <v>2.66705447235996</v>
-      </c>
-    </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="33" t="n">
-        <f aca="false">$D$14/$B$32</f>
-        <v>20.5263157894737</v>
-      </c>
-      <c r="C34" s="33" t="n">
-        <f aca="false">$D$14/$C$32</f>
-        <v>19.4173892676639</v>
+        <v>70</v>
+      </c>
+      <c r="B34" s="34" t="n">
+        <f aca="false">$F$22/($F$15*$B$33)</f>
+        <v>3.06103014860152</v>
+      </c>
+      <c r="C34" s="34" t="n">
+        <f aca="false">$F$22/($F$15*$C$33)</f>
+        <v>2.81936987371192</v>
+      </c>
+      <c r="D34" s="34" t="n">
+        <f aca="false">$F$22/($F$15*$D$33)</f>
+        <v>2.66705447235996</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="B35" s="37" t="n">
-        <f aca="false">$D$21/($D$14/$B$32)-1</f>
-        <v>-0.0616923076923076</v>
-      </c>
-      <c r="C35" s="37" t="n">
-        <f aca="false">$D$21/($D$14/$C$32)-1</f>
-        <v>-0.00810558337654377</v>
+        <v>71</v>
+      </c>
+      <c r="B35" s="33" t="n">
+        <f aca="false">$D$15/$B$33</f>
+        <v>22.2857142857143</v>
+      </c>
+      <c r="C35" s="33" t="n">
+        <f aca="false">$D$15/$C$33</f>
+        <v>20.5263157894737</v>
+      </c>
+      <c r="D35" s="33" t="n">
+        <f aca="false">$D$15/$D$33</f>
+        <v>19.4173892676639</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="34" t="n">
-        <f aca="false">$F$21/($F$15*$B$32)</f>
-        <v>2.41295112567732</v>
-      </c>
-      <c r="C36" s="34" t="n">
-        <f aca="false">$F$21/($F$15*$C$32)</f>
-        <v>2.28259234495221</v>
+        <v>72</v>
+      </c>
+      <c r="B36" s="37" t="n">
+        <f aca="false">$D$22/($D$15/$B$33)-1</f>
+        <v>-0.135769230769231</v>
+      </c>
+      <c r="C36" s="37" t="n">
+        <f aca="false">$D$22/($D$15/$C$33)-1</f>
+        <v>-0.0616923076923076</v>
+      </c>
+      <c r="D36" s="37" t="n">
+        <f aca="false">$D$22/($D$15/$D$33)-1</f>
+        <v>-0.00810558337654377</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="B37" s="33" t="n">
-        <f aca="false">$D$15/$B$32</f>
-        <v>24.8245614035088</v>
-      </c>
-      <c r="C37" s="33" t="n">
-        <f aca="false">$D$15/$C$32</f>
-        <v>23.4834237724311</v>
+        <v>73</v>
+      </c>
+      <c r="B37" s="34" t="n">
+        <f aca="false">$F$22/($F$16*$B$33)</f>
+        <v>2.61977550787824</v>
+      </c>
+      <c r="C37" s="34" t="n">
+        <f aca="false">$F$22/($F$16*$C$33)</f>
+        <v>2.41295112567732</v>
+      </c>
+      <c r="D37" s="34" t="n">
+        <f aca="false">$F$22/($F$16*$D$33)</f>
+        <v>2.28259234495221</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="B38" s="37" t="n">
-        <f aca="false">$D$21/($D$15/$B$32)-1</f>
-        <v>-0.224155477031802</v>
-      </c>
-      <c r="C38" s="37" t="n">
-        <f aca="false">$D$21/($D$15/$C$32)-1</f>
-        <v>-0.179847019470358</v>
+        <v>74</v>
+      </c>
+      <c r="B38" s="33" t="n">
+        <f aca="false">$D$16/$B$33</f>
+        <v>26.952380952381</v>
+      </c>
+      <c r="C38" s="33" t="n">
+        <f aca="false">$D$16/$C$33</f>
+        <v>24.8245614035088</v>
+      </c>
+      <c r="D38" s="33" t="n">
+        <f aca="false">$D$16/$D$33</f>
+        <v>23.4834237724311</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="B39" s="33" t="n">
-        <f aca="false">$D$16/$B$32</f>
+        <v>75</v>
+      </c>
+      <c r="B39" s="37" t="n">
+        <f aca="false">$D$22/($D$16/$B$33)-1</f>
+        <v>-0.285406360424028</v>
+      </c>
+      <c r="C39" s="37" t="n">
+        <f aca="false">$D$22/($D$16/$C$33)-1</f>
+        <v>-0.224155477031802</v>
+      </c>
+      <c r="D39" s="37" t="n">
+        <f aca="false">$D$22/($D$16/$D$33)-1</f>
+        <v>-0.179847019470358</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" s="33" t="n">
+        <f aca="false">$D$17/$B$33</f>
+        <v>18.4761904761905</v>
+      </c>
+      <c r="C40" s="33" t="n">
+        <f aca="false">$D$17/$C$33</f>
         <v>17.0175438596491</v>
       </c>
-      <c r="C39" s="33" t="n">
-        <f aca="false">$D$16/$C$32</f>
+      <c r="D40" s="33" t="n">
+        <f aca="false">$D$17/$D$33</f>
         <v>16.0981774270376</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="23" t="s">
-        <v>74</v>
-      </c>
-    </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="24" t="s">
-        <v>75</v>
-      </c>
-      <c r="B42" s="34" t="n">
+      <c r="A42" s="23" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="34" t="n">
         <f aca="false">MIN(Monthly!$C$56:$C$122)</f>
         <v>19.26</v>
       </c>
-      <c r="C42" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A$56:$A$122,MATCH(B42,Monthly!$C$56:$C$122,0))</f>
+      <c r="C43" s="32" t="n">
+        <f aca="false">INDEX(Monthly!$A$56:$A$122,MATCH(B43,Monthly!$C$56:$C$122,0))</f>
         <v>46293</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="B43" s="33" t="n">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="33" t="n">
         <f aca="false">MEDIAN(Monthly!$C$56:$C$122)</f>
         <v>22</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="B44" s="34" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="34" t="n">
         <f aca="false">SMALL(Monthly!$C$56:$C$122,2)</f>
         <v>19.5</v>
       </c>
-      <c r="C44" s="32" t="n">
-        <f aca="false">INDEX(Monthly!$A$56:$A$122,MATCH(B44,Monthly!$C$56:$C$122,0))</f>
+      <c r="C45" s="32" t="n">
+        <f aca="false">INDEX(Monthly!$A$56:$A$122,MATCH(B45,Monthly!$C$56:$C$122,0))</f>
         <v>44742</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="24" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="33" t="n">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="33" t="n">
         <f aca="false">MEDIAN(Monthly!$C$2:$C$55)</f>
         <v>26.35</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="B46" s="33" t="n">
-        <f aca="false">B45/$B$11</f>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B47" s="33" t="n">
+        <f aca="false">B46/$B$11</f>
         <v>21.8653080001258</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="22" t="s">
-        <v>80</v>
-      </c>
-    </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="19" t="n">
+      <c r="A49" s="22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="19" t="n">
         <f aca="false">Monthly!A2</f>
         <v>42643</v>
       </c>
-      <c r="B49" s="40" t="n">
+      <c r="B50" s="40" t="n">
         <f aca="false">Monthly!C122</f>
         <v>19.26</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="19" t="n">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="19" t="n">
         <f aca="false">Monthly!A122</f>
         <v>46293</v>
       </c>
-      <c r="B50" s="40" t="n">
+      <c r="B51" s="40" t="n">
         <f aca="false">Monthly!C122</f>
         <v>19.26</v>
       </c>
@@ -43332,7 +43521,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="14"/>
@@ -43345,7 +43534,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="41" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43353,22 +43542,22 @@
         <v>19</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E2" s="42" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F2" s="42" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="G2" s="42" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43386,13 +43575,13 @@
         <v>0</v>
       </c>
       <c r="E3" s="24" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43410,13 +43599,13 @@
         <v>-0.04</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43434,13 +43623,13 @@
         <v>0</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43458,13 +43647,13 @@
         <v>0</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43482,13 +43671,13 @@
         <v>0</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43506,13 +43695,13 @@
         <v>0</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43530,13 +43719,13 @@
         <v>0.01</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43554,13 +43743,13 @@
         <v>-0.02</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43578,13 +43767,13 @@
         <v>0</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43602,13 +43791,13 @@
         <v>-0.02</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43626,13 +43815,13 @@
         <v>0.02</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43650,13 +43839,13 @@
         <v>0</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43674,13 +43863,13 @@
         <v>0.05</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43698,13 +43887,13 @@
         <v>0</v>
       </c>
       <c r="E16" s="24" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43722,13 +43911,13 @@
         <v>0</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43746,13 +43935,13 @@
         <v>0.01</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43770,13 +43959,13 @@
         <v>0</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43794,13 +43983,13 @@
         <v>0</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43818,13 +44007,13 @@
         <v>0.04</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43842,13 +44031,13 @@
         <v>0</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43866,13 +44055,13 @@
         <v>-0.04</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F23" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43890,13 +44079,13 @@
         <v>-0.03</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="F24" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G24" s="24" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43914,13 +44103,13 @@
         <v>0</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F25" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G25" s="24" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43938,13 +44127,13 @@
         <v>0.02</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F26" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G26" s="24" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43962,13 +44151,13 @@
         <v>0.08</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F27" s="24" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G27" s="24" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43986,18 +44175,18 @@
         <v>-0.04</v>
       </c>
       <c r="E28" s="24" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F28" s="24" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="G28" s="24" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="24" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D29" s="40" t="n">
         <f aca="false">SUMPRODUCT(MAX(ABS(D3:D28)))</f>
@@ -44006,266 +44195,280 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="41" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="42" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B33" s="42" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C33" s="42"/>
       <c r="D33" s="42"/>
       <c r="E33" s="42" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F33" s="42"/>
       <c r="G33" s="42" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B34" s="39" t="n">
         <f aca="false">Summary!B9</f>
         <v>1.20510536599111</v>
       </c>
       <c r="E34" s="24" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="G34" s="24" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B35" s="28" t="n">
         <v>1.16</v>
       </c>
       <c r="E35" s="24" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G35" s="24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B36" s="28" t="n">
         <v>1.14</v>
       </c>
       <c r="E36" s="24" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G36" s="24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="24" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B37" s="28" t="n">
         <v>1.137</v>
       </c>
       <c r="E37" s="24" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="G37" s="24" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="41" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="B40" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="C40" s="36" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="D40" s="36" t="s">
+      <c r="B38" s="28" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E38" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="E40" s="36" t="s">
+      <c r="G38" s="24" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="24" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="B41" s="44" t="n">
-        <v>393</v>
-      </c>
-      <c r="E41" s="24" t="s">
+    </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="36" t="s">
         <v>159</v>
+      </c>
+      <c r="B41" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="C41" s="36" t="s">
+        <v>161</v>
+      </c>
+      <c r="D41" s="36" t="s">
+        <v>162</v>
+      </c>
+      <c r="E41" s="36" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B42" s="44" t="n">
+        <v>393</v>
+      </c>
+      <c r="E42" s="24" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24" t="s">
+        <v>166</v>
+      </c>
+      <c r="B43" s="44" t="n">
         <v>481</v>
       </c>
-      <c r="C42" s="10" t="n">
+      <c r="C43" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2019,5,31),Monthly!$A:$A,1))</f>
         <v>404.162711864407</v>
       </c>
-      <c r="D42" s="40" t="n">
-        <f aca="false">C42/B42</f>
+      <c r="D43" s="40" t="n">
+        <f aca="false">C43/B43</f>
         <v>0.84025511822122</v>
       </c>
-      <c r="E42" s="24" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B43" s="44" t="n">
+      <c r="E43" s="24" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="44" t="n">
         <v>539</v>
       </c>
-      <c r="C43" s="10" t="n">
+      <c r="C44" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2021,5,31),Monthly!$A:$A,1))</f>
         <v>533.657534246575</v>
       </c>
-      <c r="D43" s="40" t="n">
-        <f aca="false">C43/B43</f>
+      <c r="D44" s="40" t="n">
+        <f aca="false">C44/B44</f>
         <v>0.9900881896968</v>
       </c>
-      <c r="E43" s="24" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="24" t="s">
-        <v>164</v>
-      </c>
-      <c r="B44" s="44" t="n">
+      <c r="E44" s="24" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B45" s="44" t="n">
         <v>737</v>
       </c>
-      <c r="C44" s="10" t="n">
+      <c r="C45" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2022,5,31),Monthly!$A:$A,1))</f>
         <v>812.968137254902</v>
       </c>
-      <c r="D44" s="40" t="n">
-        <f aca="false">C44/B44</f>
+      <c r="D45" s="40" t="n">
+        <f aca="false">C45/B45</f>
         <v>1.10307752680448</v>
       </c>
-      <c r="E44" s="24" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="24" t="s">
-        <v>166</v>
-      </c>
-      <c r="B45" s="44" t="n">
+      <c r="E45" s="24" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="B46" s="44" t="n">
         <v>806</v>
       </c>
-      <c r="C45" s="10" t="n">
+      <c r="C46" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2023,5,31),Monthly!$A:$A,1))</f>
         <v>858.074074074074</v>
       </c>
-      <c r="D45" s="40" t="n">
-        <f aca="false">C45/B45</f>
+      <c r="D46" s="40" t="n">
+        <f aca="false">C46/B46</f>
         <v>1.06460803234997</v>
       </c>
-      <c r="E45" s="24" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="B46" s="44" t="n">
+      <c r="E46" s="24" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="B47" s="44" t="n">
         <v>1005</v>
       </c>
-      <c r="C46" s="10" t="n">
+      <c r="C47" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2024,5,31),Monthly!$A:$A,1))</f>
         <v>1052.83644859813</v>
       </c>
-      <c r="D46" s="40" t="n">
-        <f aca="false">C46/B46</f>
+      <c r="D47" s="40" t="n">
+        <f aca="false">C47/B47</f>
         <v>1.04759845631655</v>
       </c>
-      <c r="E46" s="24" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="B47" s="44" t="n">
+      <c r="E47" s="24" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="B48" s="44" t="n">
         <v>1013</v>
       </c>
-      <c r="C47" s="10" t="n">
+      <c r="C48" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2025,5,31),Monthly!$A:$A,1))</f>
         <v>1109.89686098655</v>
       </c>
-      <c r="D47" s="40" t="n">
-        <f aca="false">C47/B47</f>
+      <c r="D48" s="40" t="n">
+        <f aca="false">C48/B48</f>
         <v>1.09565336721278</v>
       </c>
-      <c r="E47" s="24" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="B48" s="44" t="n">
+      <c r="E48" s="24" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="B49" s="44" t="n">
         <v>1065</v>
       </c>
-      <c r="C48" s="10" t="n">
+      <c r="C49" s="10" t="n">
         <f aca="false">INDEX(Monthly!$E:$E,MATCH(DATE(2026,5,31),Monthly!$A:$A,1))</f>
         <v>1159.98768472906</v>
       </c>
-      <c r="D48" s="40" t="n">
-        <f aca="false">C48/B48</f>
+      <c r="D49" s="40" t="n">
+        <f aca="false">C49/B49</f>
         <v>1.08919031429959</v>
       </c>
-      <c r="E48" s="24" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="B49" s="34" t="n">
-        <f aca="false">B48/B41</f>
+      <c r="E49" s="24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="24" t="s">
+        <v>180</v>
+      </c>
+      <c r="B50" s="34" t="n">
+        <f aca="false">B49/B42</f>
         <v>2.70992366412214</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="22" t="s">
-        <v>175</v>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="22" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -44284,7 +44487,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
@@ -44292,37 +44495,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="45" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="46" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="46" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="46" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="46" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="46" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="46" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -44330,22 +44533,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="45" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="46" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="46" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="46" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -44353,52 +44556,57 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="45" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="46" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="46" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="46" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="46" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="46" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="46" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="46" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="46" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="46" t="s">
-        <v>196</v>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="46" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>